<commit_message>
chore: update AI Audit Log
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example.xlsx
+++ b/AI_AuditLog_Example.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\Downloads\labnopswr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29897A62-9558-4752-90E8-A724E450DAE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724A4331-34AF-45C2-9810-CD4B920F559C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="152">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -34,12 +34,21 @@
     <t>Student Name:</t>
   </si>
   <si>
+    <t>Nguyễn Thành Đạt</t>
+  </si>
+  <si>
     <t>Student ID:</t>
   </si>
   <si>
+    <t>DE190465</t>
+  </si>
+  <si>
     <t>Course:</t>
   </si>
   <si>
+    <t>SWR302</t>
+  </si>
+  <si>
     <t>Assignment:</t>
   </si>
   <si>
@@ -52,15 +61,9 @@
     <t>Total Prompts Used (all AI tools):</t>
   </si>
   <si>
-    <t>[e.g., ~150]</t>
-  </si>
-  <si>
     <t>Core Prompts Logged:</t>
   </si>
   <si>
-    <t>[e.g., 18]</t>
-  </si>
-  <si>
     <t>Selection Ratio:</t>
   </si>
   <si>
@@ -70,9 +73,6 @@
     <t>Hallucination Detected:</t>
   </si>
   <si>
-    <t>[Count]</t>
-  </si>
-  <si>
     <t>AI TOOLS USED</t>
   </si>
   <si>
@@ -184,12 +184,114 @@
     <t>001</t>
   </si>
   <si>
+    <t>DECISION</t>
+  </si>
+  <si>
+    <t>Chưa rõ tiêu chí phân biệt rõ ràng giữa các mức độ ưu tiên trong phương pháp MoSCoW, đặc biệt là ranh giới giữa Must Have và Should Have khi làm việc với khách hàng thực tế.</t>
+  </si>
+  <si>
+    <t>Thế nào là phương pháp MoSCoW? Làm thế nào để phân biệt chính xác giữa yêu cầu Must Have và Should Have khi phân tích dự án phần mềm?</t>
+  </si>
+  <si>
+    <t>AI định nghĩa MoSCoW (Must, Should, Could, Won't). Phân biệt Must và Should bằng câu hỏi cốt lõi: "Nếu thiếu tính năng này, hệ thống có thể vận hành và bàn giao được không?" (Must: Bắt buộc, hệ thống không chạy được nếu thiếu; Should: Quan trọng nhưng vẫn có thể vận hành tạm thời bằng cách khác).</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Lý thuyết của AI rất rõ ràng nhưng trong thực tế ranh giới này dễ bị nhầm lẫn do khách hàng (giám đốc) luôn muốn mọi thứ là "Must Have" để tối đa hóa quyền lợi.
+Contextualization: Với dự án phòng khám 8 tuần và 3 dev, nếu áp dụng máy móc định nghĩa của AI thì danh sách "Must Have" sẽ quá dài và chắc chắn sẽ bị trễ deadline.
+Creative Synthesis: Tôi tự xây dựng một bộ quy tắc lọc (Checklist) gồm 3 câu hỏi thực tế để tự phản biện yêu cầu của khách hàng: (1) Có giải pháp thay thế thủ công tạm thời không? (2) Thiếu nó hệ thống có bị lỗi vận hành nghiêm trọng không? (3) Việc thiếu nó có vi phạm pháp luật y tế hay không?
+Decision: Quyết định dùng bộ quy tắc lọc này làm tiêu chuẩn chung để đánh giá và phân loại cho 10 yêu cầu chi tiết ở bài tập tiếp theo nhằm thu hẹp phạm vi MVP.</t>
+  </si>
+  <si>
+    <t>Sơ đồ tư duy tiêu chuẩn lọc MoSCoW tự vẽ trong ghi chú cá nhân.</t>
+  </si>
+  <si>
     <t>002</t>
   </si>
   <si>
+    <t>Cần phân loại độ ưu tiên cho 10 requirements với nguồn lực giới hạn (8 tuần, 3 dev) của app đặt lịch khám trực tuyến và điều chỉnh khi deadline bị rút xuống 5 tuần.</t>
+  </si>
+  <si>
+    <t>Phân loại MoSCoW cho 10 requirements của ứng dụng đặt lịch khám trực tuyến với deadline 8 tuần, nhóm 3 dev: [liệt kê R01 - R10]. Đề xuất hạ cấp tính năng nào nếu deadline rút xuống còn 5 tuần?</t>
+  </si>
+  <si>
+    <t>AI đề xuất phân loại: Must Have (R01, R02, R03, R06, R07), Should Have (R04, R08), Could Have (R05, R09), Won't Have (R10). Khi rút ngắn hạn, AI khuyên hạ cấp R08 và R09.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đề xuất quá nhiều Must Have (5/10 tính năng), đặc biệt xếp R07 (Thanh toán trực tuyến VNPay/MoMo) và R03 (SMS nhắc lịch) vào nhóm ưu tiên cao là thiếu thực tế với lực lượng 3 dev.
+Contextualization: Với 8 tuần và 3 dev, tích hợp API thanh toán rất phức tạp (thủ tục ngân hàng, xử lý lỗi giao dịch). MVP chỉ cần đặt lịch trước, trả tiền mặt tại quầy sau.
+Creative Synthesis: Tôi hạ cấp R07 xuống Should Have và SMS tự động R03 xuống Should Have. Tối giản hóa nhóm Must Have chỉ còn R01, R02, R06. Khi hạn rút còn 5 tuần, tôi chủ động hạ cấp R07 và R03 xuống Could Have thay vì hạ R08/R09 vốn dĩ đã là Could Have sẵn.
+Decision: Quyết định chọn giữ lại đúng 3 module cốt lõi (R01, R02, R06) cho nhóm Must Have để giảm tải 40% khối lượng phát triển cho đội ngũ dev, đảm bảo ra mắt đúng hạn.</t>
+  </si>
+  <si>
     <t>003</t>
   </si>
   <si>
+    <t>Chưa phân biệt rõ bản chất và sự khác biệt cốt lõi giữa hai khái niệm Validation (Thẩm định) và Verification (Kiểm định) để chuẩn bị làm bài tập 2.</t>
+  </si>
+  <si>
+    <t>Verification và Validation là gì? Sự khác biệt cốt lõi giữa hai khái niệm này là gì và làm thế nào để nhớ lâu?</t>
+  </si>
+  <si>
+    <t>AI định nghĩa: Verification đảm bảo sản phẩm xây dựng đúng theo tài liệu đặc tả kỹ thuật ("Are we building the product right?"). Validation đảm bảo sản phẩm đáp ứng đúng nhu cầu thực tế của người dùng cuối ("Are we building the right product?").</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Phân biệt của AI mang tính lý thuyết giáo khoa. Tôi nhận thấy điểm mấu chốt là: Một phần mềm có thể vượt qua tất cả các bài kiểm tra kỹ thuật (Verification PASS) nhưng vẫn bị người dùng từ chối nếu nó không giải quyết được vấn đề thực tế của họ (Validation FAIL).
+Contextualization: Trong ngành phần mềm, nếu chỉ tập trung vào Verification mà bỏ qua Validation thì sản phẩm làm ra sẽ bị lãng phí tài nguyên và thất bại về mặt thương mại.
+Creative Synthesis: Tôi tự hệ thống hóa hai khái niệm này bằng cách ví von thực tế: Verification giống như việc kiểm tra xem cây cầu có được xây đúng bản vẽ kỹ thuật không, còn Validation là kiểm tra xem cây cầu đó có được xây đúng con sông cần đi qua hay không.
+Decision: Quyết định sử dụng quy tắc ví von này làm hệ quy chiếu tiêu chuẩn để phân tích 5 tình huống thực tế trong Bài tập 2a của môn học.</t>
+  </si>
+  <si>
+    <t>Ghi chú sơ đồ tư duy phân biệt V&amp;V trong file học tập cá nhân.</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t>PROBLEM-SOLVING</t>
+  </si>
+  <si>
+    <t>Phân tích sự giao thoa giữa hai khái niệm và giải quyết tình huống TH5: Tại sao 200 automated test cases đều PASS nhưng khách hàng vẫn từ chối nghiệm thu sản phẩm.</t>
+  </si>
+  <si>
+    <t>Có trường hợp nào một hoạt động kiểm thử thuộc về cả hai nhóm Verification và Validation không? Tại sao hệ thống phần mềm pass 100% test kỹ thuật nhưng khách hàng vẫn từ chối nghiệm thu?</t>
+  </si>
+  <si>
+    <t>AI khẳng định có sự giao thoa (như quy trình UAT) và giải thích tình huống TH5 do dự án đạt Verification nhưng hỏng Validation vì tài liệu SRS ghi sai nhu cầu khách hàng (bắt nhập cả CMND lẫn BHYT).</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI giải thích đúng bản chất nhưng lại đổ lỗi cho khâu kiểm thử. Tôi nhận thấy lỗi gốc rễ là ở BA khi phân tích yêu cầu đã không thực hiện Validation cho tài liệu SRS với khách hàng trước khi bàn giao cho Dev/QA.
+Contextualization: Trong thực tế dự án, việc chỉ tập trung chạy test case kỹ thuật (Verification) mà thiếu đi các buổi demo prototype sớm (Validation) cho khách hàng là nguyên nhân hàng đầu gây hỏng dự án.
+Creative Synthesis: Tôi đề xuất quy trình bắt buộc phải Validation tài liệu SRS thông qua Mockup trực quan trước khi đóng băng yêu cầu.
+Decision: Quyết định chọn bổ sung hoạt động User Acceptance Testing (UAT) và chạy thử nghiệm giới hạn (Pilot Run) trước khi bàn giao chính thức để tránh lỗi TH5 lập lại.</t>
+  </si>
+  <si>
+    <t>Phần phân tích TH5 trong file README.md.</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>VERIFICATION</t>
+  </si>
+  <si>
+    <t>Thiết kế Acceptance Criteria định dạng Given-When-Then cho User Story đặt lịch trực tuyến sao cho bao quát được các trường hợp lỗi/lạm dụng hệ thống.</t>
+  </si>
+  <si>
+    <t>Viết Acceptance Criteria dạng Given-When-Then cho user story: Bệnh nhân muốn đặt lịch khám trực tuyến để không phải chờ lấy số. Làm thế nào để không bỏ sót các tiêu chí quan trọng?</t>
+  </si>
+  <si>
+    <t>AI cung cấp các AC cơ bản cho luồng đặt lịch thành công, đặt trùng giờ và điền thiếu thông tin bắt buộc.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI chỉ tập trung vào các luồng chạy đúng thông thường (Happy Path) mà bỏ qua các kịch bản biên hoặc hành vi cố tình spam/lạm dụng hệ thống từ người dùng (như đặt hàng loạt rồi hủy sát nút).
+Contextualization: Nếu không giới hạn số lượt đặt lịch và thời gian hủy lịch tối đa trong ngày, phòng khám dễ bị đối thủ hoặc cò mồi spam đặt lịch ảo rồi hủy sát giờ.
+Creative Synthesis: Tôi tự thiết kế thêm AC bổ sung: giới hạn đặt tối đa 2 lịch hẹn/ngày và chỉ cho phép hủy trước giờ khám tối thiểu 24 giờ.
+Decision: Quyết định đưa các ràng buộc nghiệp vụ (anti-spam) này vào AC để làm căn cứ cho Dev viết mã kiểm tra điều kiện và QA viết Negative Test Cases.</t>
+  </si>
+  <si>
+    <t>Bảng Acceptance Criteria 4 và Test Case hủy lịch hẹn trong file README.md.</t>
+  </si>
+  <si>
     <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
   </si>
   <si>
@@ -229,6 +331,21 @@
     <t>Used real paper 'Jones et al. 2022'</t>
   </si>
   <si>
+    <t>Context Misunderstanding</t>
+  </si>
+  <si>
+    <t>AI khẳng định việc tích hợp ví điện tử MoMo/VNPay (R07) và hệ thống nhắc lịch SMS (R03) là đơn giản, có thể hoàn thành trong 1-2 ngày và khuyên nên để vào Must Have.</t>
+  </si>
+  <si>
+    <t>Thực tế tại Việt Nam, đăng ký tích hợp cổng thanh toán doanh nghiệp cần giấy phép kinh doanh, mã số thuế, ký hợp đồng và duyệt hồ sơ mất ít nhất 7-10 ngày làm việc. Hệ thống SMS Brandname cũng cần đăng ký mẫu tin nhắn duyệt với nhà mạng.</t>
+  </si>
+  <si>
+    <t>Tra cứu tài liệu tích hợp (API Integration Guide) của VNPay và quy trình đăng ký dịch vụ eSMS.</t>
+  </si>
+  <si>
+    <t>Hạ cấp cả 2 tính năng xuống Should/Could Have để tránh làm trễ deadline dự án.</t>
+  </si>
+  <si>
     <t>HALLUCINATION TYPES REFERENCE:</t>
   </si>
   <si>
@@ -274,9 +391,6 @@
     <t>Old API syntax, deprecated methods</t>
   </si>
   <si>
-    <t>Context Misunderstanding</t>
-  </si>
-  <si>
     <t>AI không hiểu đúng bối cảnh</t>
   </si>
   <si>
@@ -380,15 +494,6 @@
   </si>
   <si>
     <t>Tôi có evidence?</t>
-  </si>
-  <si>
-    <t>Nguyễn Thành Đạt</t>
-  </si>
-  <si>
-    <t>DE190465</t>
-  </si>
-  <si>
-    <t>SWR302</t>
   </si>
 </sst>
 </file>
@@ -528,7 +633,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -564,6 +669,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -894,16 +1002,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-    </row>
-    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+    </row>
+    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -913,75 +1021,75 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>119</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>120</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="C11" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="4" t="e">
+        <v>13</v>
+      </c>
+      <c r="C12" s="4">
         <f>C11/C10</f>
-        <v>#VALUE!</v>
+        <v>0.2</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="C13" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1050,7 +1158,7 @@
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
     </row>
-    <row r="22" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>33</v>
       </c>
@@ -1071,7 +1179,7 @@
         <v>37</v>
       </c>
       <c r="B24" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>38</v>
@@ -1082,7 +1190,7 @@
         <v>39</v>
       </c>
       <c r="B25" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>38</v>
@@ -1093,7 +1201,7 @@
         <v>40</v>
       </c>
       <c r="B26" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>38</v>
@@ -1104,7 +1212,7 @@
         <v>41</v>
       </c>
       <c r="B27" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>38</v>
@@ -1133,28 +1241,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -1182,55 +1290,133 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+    <row r="4" spans="1:8" ht="241.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="225.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>63</v>
+      </c>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+    <row r="6" spans="1:8" ht="240.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="205.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="215.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7"/>
@@ -1402,74 +1588,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="A1" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="A2" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
@@ -1623,75 +1819,75 @@
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
     </row>
-    <row r="30" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>68</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>84</v>
+        <v>117</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1715,216 +1911,216 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
+      <c r="A1" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-    </row>
-    <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A2" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>89</v>
+        <v>122</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D7" s="13"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D10" s="13"/>
     </row>
-    <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>89</v>
+        <v>122</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>107</v>
+        <v>140</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>108</v>
+        <v>141</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>109</v>
+        <v>142</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D18" s="13"/>
     </row>
-    <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="17" t="s">
         <v>44</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>118</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1937,7 +2133,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -1945,7 +2141,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>

</xml_diff>

<commit_message>
chore: update audit log
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Example.xlsx
+++ b/AI_AuditLog_Example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\Downloads\labnopswr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724A4331-34AF-45C2-9810-CD4B920F559C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC08EF6E-0C61-453E-8420-BEE8D9498C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,12 @@
     <sheet name="3. Hallucination Detection" sheetId="3" r:id="rId3"/>
     <sheet name="4. Self-Assessment Checklist" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="172">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -198,11 +198,11 @@
   <si>
     <t>Critical Thinking: Lý thuyết của AI rất rõ ràng nhưng trong thực tế ranh giới này dễ bị nhầm lẫn do khách hàng (giám đốc) luôn muốn mọi thứ là "Must Have" để tối đa hóa quyền lợi.
 Contextualization: Với dự án phòng khám 8 tuần và 3 dev, nếu áp dụng máy móc định nghĩa của AI thì danh sách "Must Have" sẽ quá dài và chắc chắn sẽ bị trễ deadline.
-Creative Synthesis: Tôi tự xây dựng một bộ quy tắc lọc (Checklist) gồm 3 câu hỏi thực tế để tự phản biện yêu cầu của khách hàng: (1) Có giải pháp thay thế thủ công tạm thời không? (2) Thiếu nó hệ thống có bị lỗi vận hành nghiêm trọng không? (3) Việc thiếu nó có vi phạm pháp luật y tế hay không?
+Creative Synthesis: Em tự xây dựng một bộ quy tắc lọc (Checklist) gồm 3 câu hỏi thực tế để tự phản biện yêu cầu của khách hàng: (1) Có giải pháp thay thế thủ công tạm thời không? (2) Thiếu nó hệ thống có bị lỗi vận hành nghiêm trọng không? (3) Việc thiếu nó có vi phạm pháp luật y tế hay không?
 Decision: Quyết định dùng bộ quy tắc lọc này làm tiêu chuẩn chung để đánh giá và phân loại cho 10 yêu cầu chi tiết ở bài tập tiếp theo nhằm thu hẹp phạm vi MVP.</t>
   </si>
   <si>
-    <t>Sơ đồ tư duy tiêu chuẩn lọc MoSCoW tự vẽ trong ghi chú cá nhân.</t>
+    <t>Sơ đồ tư duy tiêu chuẩn lọc MoSCoW tự vẽ trong ghi chú cá nhân hoặc file Bài làm (Word).</t>
   </si>
   <si>
     <t>002</t>
@@ -219,7 +219,7 @@
   <si>
     <t>Critical Thinking: AI đề xuất quá nhiều Must Have (5/10 tính năng), đặc biệt xếp R07 (Thanh toán trực tuyến VNPay/MoMo) và R03 (SMS nhắc lịch) vào nhóm ưu tiên cao là thiếu thực tế với lực lượng 3 dev.
 Contextualization: Với 8 tuần và 3 dev, tích hợp API thanh toán rất phức tạp (thủ tục ngân hàng, xử lý lỗi giao dịch). MVP chỉ cần đặt lịch trước, trả tiền mặt tại quầy sau.
-Creative Synthesis: Tôi hạ cấp R07 xuống Should Have và SMS tự động R03 xuống Should Have. Tối giản hóa nhóm Must Have chỉ còn R01, R02, R06. Khi hạn rút còn 5 tuần, tôi chủ động hạ cấp R07 và R03 xuống Could Have thay vì hạ R08/R09 vốn dĩ đã là Could Have sẵn.
+Creative Synthesis: Em hạ cấp R07 xuống Should Have và SMS tự động R03 xuống Should Have. Tối giản hóa nhóm Must Have chỉ còn R01, R02, R06. Khi hạn rút còn 5 tuần, em chủ động hạ cấp R07 và R03 xuống Could Have thay vì hạ R08/R09 vốn dĩ đã là Could Have sẵn.
 Decision: Quyết định chọn giữ lại đúng 3 module cốt lõi (R01, R02, R06) cho nhóm Must Have để giảm tải 40% khối lượng phát triển cho đội ngũ dev, đảm bảo ra mắt đúng hạn.</t>
   </si>
   <si>
@@ -235,9 +235,9 @@
     <t>AI định nghĩa: Verification đảm bảo sản phẩm xây dựng đúng theo tài liệu đặc tả kỹ thuật ("Are we building the product right?"). Validation đảm bảo sản phẩm đáp ứng đúng nhu cầu thực tế của người dùng cuối ("Are we building the right product?").</t>
   </si>
   <si>
-    <t>Critical Thinking: Phân biệt của AI mang tính lý thuyết giáo khoa. Tôi nhận thấy điểm mấu chốt là: Một phần mềm có thể vượt qua tất cả các bài kiểm tra kỹ thuật (Verification PASS) nhưng vẫn bị người dùng từ chối nếu nó không giải quyết được vấn đề thực tế của họ (Validation FAIL).
+    <t>Critical Thinking: Phân biệt của AI mang tính lý thuyết giáo khoa. Em nhận thấy điểm mấu chốt là: Một phần mềm có thể vượt qua tất cả các bài kiểm tra kỹ thuật (Verification PASS) nhưng vẫn bị người dùng từ chối nếu nó không giải quyết được vấn đề thực tế của họ (Validation FAIL).
 Contextualization: Trong ngành phần mềm, nếu chỉ tập trung vào Verification mà bỏ qua Validation thì sản phẩm làm ra sẽ bị lãng phí tài nguyên và thất bại về mặt thương mại.
-Creative Synthesis: Tôi tự hệ thống hóa hai khái niệm này bằng cách ví von thực tế: Verification giống như việc kiểm tra xem cây cầu có được xây đúng bản vẽ kỹ thuật không, còn Validation là kiểm tra xem cây cầu đó có được xây đúng con sông cần đi qua hay không.
+Creative Synthesis: Em tự hệ thống hóa hai khái niệm này bằng cách ví von thực tế: Verification giống như việc kiểm tra xem cây cầu có được xây đúng bản vẽ kỹ thuật không, còn Validation là kiểm tra xem cây cầu đó có được xây đúng con sông cần đi qua hay không.
 Decision: Quyết định sử dụng quy tắc ví von này làm hệ quy chiếu tiêu chuẩn để phân tích 5 tình huống thực tế trong Bài tập 2a của môn học.</t>
   </si>
   <si>
@@ -259,13 +259,13 @@
     <t>AI khẳng định có sự giao thoa (như quy trình UAT) và giải thích tình huống TH5 do dự án đạt Verification nhưng hỏng Validation vì tài liệu SRS ghi sai nhu cầu khách hàng (bắt nhập cả CMND lẫn BHYT).</t>
   </si>
   <si>
-    <t>Critical Thinking: AI giải thích đúng bản chất nhưng lại đổ lỗi cho khâu kiểm thử. Tôi nhận thấy lỗi gốc rễ là ở BA khi phân tích yêu cầu đã không thực hiện Validation cho tài liệu SRS với khách hàng trước khi bàn giao cho Dev/QA.
+    <t>Critical Thinking: AI giải thích đúng bản chất nhưng lại đổ lỗi cho khâu kiểm thử. Em nhận thấy lỗi gốc rễ là ở BA khi phân tích yêu cầu đã không thực hiện Validation cho tài liệu SRS với khách hàng trước khi bàn giao cho Dev/QA.
 Contextualization: Trong thực tế dự án, việc chỉ tập trung chạy test case kỹ thuật (Verification) mà thiếu đi các buổi demo prototype sớm (Validation) cho khách hàng là nguyên nhân hàng đầu gây hỏng dự án.
-Creative Synthesis: Tôi đề xuất quy trình bắt buộc phải Validation tài liệu SRS thông qua Mockup trực quan trước khi đóng băng yêu cầu.
+Creative Synthesis: Em đề xuất quy trình bắt buộc phải Validation tài liệu SRS thông qua Mockup trực quan trước khi đóng băng yêu cầu.
 Decision: Quyết định chọn bổ sung hoạt động User Acceptance Testing (UAT) và chạy thử nghiệm giới hạn (Pilot Run) trước khi bàn giao chính thức để tránh lỗi TH5 lập lại.</t>
   </si>
   <si>
-    <t>Phần phân tích TH5 trong file README.md.</t>
+    <t>Phần phân tích TH5 trong file Bài làm (Word).</t>
   </si>
   <si>
     <t>005</t>
@@ -285,11 +285,63 @@
   <si>
     <t>Critical Thinking: AI chỉ tập trung vào các luồng chạy đúng thông thường (Happy Path) mà bỏ qua các kịch bản biên hoặc hành vi cố tình spam/lạm dụng hệ thống từ người dùng (như đặt hàng loạt rồi hủy sát nút).
 Contextualization: Nếu không giới hạn số lượt đặt lịch và thời gian hủy lịch tối đa trong ngày, phòng khám dễ bị đối thủ hoặc cò mồi spam đặt lịch ảo rồi hủy sát giờ.
-Creative Synthesis: Tôi tự thiết kế thêm AC bổ sung: giới hạn đặt tối đa 2 lịch hẹn/ngày và chỉ cho phép hủy trước giờ khám tối thiểu 24 giờ.
+Creative Synthesis: Em tự thiết kế thêm AC bổ sung: giới hạn đặt tối đa 2 lịch hẹn/ngày và chỉ cho phép hủy trước giờ khám tối thiểu 24 giờ.
 Decision: Quyết định đưa các ràng buộc nghiệp vụ (anti-spam) này vào AC để làm căn cứ cho Dev viết mã kiểm tra điều kiện và QA viết Negative Test Cases.</t>
   </si>
   <si>
-    <t>Bảng Acceptance Criteria 4 và Test Case hủy lịch hẹn trong file README.md.</t>
+    <t>Bảng Acceptance Criteria 4 và Test Case hủy lịch hẹn trong file Bài làm (Word).</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>IDEA GENERATION</t>
+  </si>
+  <si>
+    <t>Elicitation / Negotiation</t>
+  </si>
+  <si>
+    <t>Cần đặt 3 câu hỏi cho tính năng SMS (R03) và Thanh toán (R07) để 'ép khéo' giám đốc hạ cấp yêu cầu mà không làm phật lòng khách hàng.</t>
+  </si>
+  <si>
+    <t>Đóng vai một BA, hãy gợi ý cho tôi 3 câu hỏi theo phương pháp thương lượng 'Games People Play' để thuyết phục Giám đốc phòng khám tạm hoãn tính năng thanh toán VNPay và tự động gửi SMS trong phiên bản đầu tiên.</t>
+  </si>
+  <si>
+    <t>AI đưa ra các câu hỏi tập trung vào việc hỏi khách hàng xem tính năng đó có 'thực sự cần thiết không' hoặc 'có ai dùng không'.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Em nhận thấy các câu hỏi AI sinh ra quá hiền và giống câu hỏi khảo sát thông thường. Để Giám đốc chịu lùi bước, ta phải lượng hóa thiệt hại.
+Creative Synthesis: Em tự sửa lại các câu hỏi của AI bằng cách đưa thẳng các thông số rủi ro vào câu hỏi: Đưa ra thời gian trễ tiến độ (trễ 1 tuần), đưa ra rào cản pháp lý (hợp đồng 2-3 tuần), và đề xuất giải pháp thay thế thủ công (lễ tân tự gọi điện / quẹt mã QR tĩnh).
+Decision: Sử dụng bộ câu hỏi đã qua chỉnh sửa sắc bén này vào bài làm để chứng minh kỹ năng thương lượng thực tế.</t>
+  </si>
+  <si>
+    <t>Các câu hỏi trong phần 1b của file Bài làm (Word).</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>TEST CASE GENERATION</t>
+  </si>
+  <si>
+    <t>Quality Assurance</t>
+  </si>
+  <si>
+    <t>Cần chuyển đổi Acceptance Criteria số 4 (Hủy lịch khám) thành một Test Case hoàn chỉnh với đầy đủ các trường thông tin chuẩn bị cho QA.</t>
+  </si>
+  <si>
+    <t>Từ Acceptance Criteria: 'Bệnh nhân hủy lịch khám hợp lệ trước 24 giờ', hãy viết cho tôi một kịch bản Test Case chi tiết gồm Pre-condition, Steps, Test Data và Expected Result.</t>
+  </si>
+  <si>
+    <t>AI sinh ra một bảng Test Case khá đầy đủ, nhưng phần Test Data chỉ ghi chung chung là 'Tài khoản hợp lệ', 'Lịch khám hợp lệ'.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Một Test Case thực tế không thể dùng data chung chung. Tester cần biết chính xác ngày giờ nào để test logic 'trước 24 giờ'.
+Contextualization: Em tự đóng vai QA, thiết kế ra các mốc thời gian giả định cụ thể: Giờ khám là 10:00 AM ngày 18/06/2026, và giờ thực hiện test là 09:00 AM ngày 17/06/2026 (đảm bảo cách nhau đúng 25 tiếng để pass điều kiện &gt; 24h).
+Decision: Quyết định cập nhật các Test Data cụ thể này vào bài làm, đồng thời bổ sung thêm Expected Result ở tầng Backend (cập nhật status = 'CANCELLED' trong DB) chứ không chỉ nhìn giao diện UI như AI gợi ý.</t>
+  </si>
+  <si>
+    <t>Test Case hủy lịch hẹn trong phần 3c của file Bài làm (Word).</t>
   </si>
   <si>
     <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
@@ -316,48 +368,51 @@
     <t>Corrective Action</t>
   </si>
   <si>
+    <t>Logical Flaw</t>
+  </si>
+  <si>
+    <t>AI cho rằng dự án pass test nhưng fail nghiệm thu (TH5) là do khâu kiểm thử (Testing) hoặc khách hàng bất hợp tác.</t>
+  </si>
+  <si>
+    <t>200 automated tests PASS nghĩa là Tester làm đúng kỹ thuật. Khách hàng từ chối là do tính năng bắt nhập giấy tờ quá rườm rà. Lỗi gốc rễ ở khâu Requirement Validation của BA.</t>
+  </si>
+  <si>
+    <t>Áp dụng kiến thức Requirement Engineering: Lỗi ở Requirement Phase sẽ lọt qua Testing Phase nếu test dựa trên đặc tả sai.</t>
+  </si>
+  <si>
+    <t>Đính chính lại nguyên nhân cốt lõi là lỗi 'dịch thuật yêu cầu' và đề xuất thêm UAT/Mockup trước khi đóng băng yêu cầu.</t>
+  </si>
+  <si>
+    <t>Context Misunderstanding</t>
+  </si>
+  <si>
+    <t>AI khẳng định việc tích hợp ví điện tử MoMo/VNPay (R07) và hệ thống nhắc lịch SMS (R03) là đơn giản, có thể hoàn thành trong 1-2 ngày và khuyên nên để vào Must Have.</t>
+  </si>
+  <si>
+    <t>Thực tế tại Việt Nam, đăng ký tích hợp cổng thanh toán doanh nghiệp cần giấy phép kinh doanh, mã số thuế, ký hợp đồng và duyệt hồ sơ mất ít nhất 7-10 ngày làm việc. Hệ thống SMS Brandname cũng cần đăng ký mẫu tin nhắn duyệt với nhà mạng.</t>
+  </si>
+  <si>
+    <t>Tra cứu tài liệu tích hợp (API Integration Guide) của VNPay và quy trình đăng ký dịch vụ eSMS.</t>
+  </si>
+  <si>
+    <t>Hạ cấp cả 2 tính năng xuống Should/Could Have để tránh làm trễ deadline dự án.</t>
+  </si>
+  <si>
+    <t>HALLUCINATION TYPES REFERENCE:</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
     <t>Fabrication</t>
   </si>
   <si>
-    <t>Paper 'Smith et al. 2023' exists</t>
-  </si>
-  <si>
-    <t>Paper NOT FOUND on Google Scholar</t>
-  </si>
-  <si>
-    <t>Searched Google Scholar, ResearchGate</t>
-  </si>
-  <si>
-    <t>Used real paper 'Jones et al. 2022'</t>
-  </si>
-  <si>
-    <t>Context Misunderstanding</t>
-  </si>
-  <si>
-    <t>AI khẳng định việc tích hợp ví điện tử MoMo/VNPay (R07) và hệ thống nhắc lịch SMS (R03) là đơn giản, có thể hoàn thành trong 1-2 ngày và khuyên nên để vào Must Have.</t>
-  </si>
-  <si>
-    <t>Thực tế tại Việt Nam, đăng ký tích hợp cổng thanh toán doanh nghiệp cần giấy phép kinh doanh, mã số thuế, ký hợp đồng và duyệt hồ sơ mất ít nhất 7-10 ngày làm việc. Hệ thống SMS Brandname cũng cần đăng ký mẫu tin nhắn duyệt với nhà mạng.</t>
-  </si>
-  <si>
-    <t>Tra cứu tài liệu tích hợp (API Integration Guide) của VNPay và quy trình đăng ký dịch vụ eSMS.</t>
-  </si>
-  <si>
-    <t>Hạ cấp cả 2 tính năng xuống Should/Could Have để tránh làm trễ deadline dự án.</t>
-  </si>
-  <si>
-    <t>HALLUCINATION TYPES REFERENCE:</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Definition</t>
-  </si>
-  <si>
-    <t>Example</t>
-  </si>
-  <si>
     <t>AI tạo ra thông tin không tồn tại</t>
   </si>
   <si>
@@ -424,7 +479,7 @@
     <t>Prompt này ảnh hưởng đến quyết định quan trọng trong project?</t>
   </si>
   <si>
-    <t>☐</t>
+    <t>☑</t>
   </si>
   <si>
     <t>2</t>
@@ -460,9 +515,15 @@
     <t>Số lượng entries nằm trong range (min-max)?</t>
   </si>
   <si>
+    <t>7</t>
+  </si>
+  <si>
     <t>Mỗi DTC component có ít nhất 1 core prompt?</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>Đã phát hiện ≥ số lượng hallucination yêu cầu?</t>
   </si>
   <si>
@@ -470,6 +531,9 @@
   </si>
   <si>
     <t>Có evidence cho ≥70% entries?</t>
+  </si>
+  <si>
+    <t>100%</t>
   </si>
   <si>
     <t>⚠️ LƯU Ý QUAN TRỌNG:</t>
@@ -1066,7 +1130,7 @@
         <v>12</v>
       </c>
       <c r="C11" s="3">
-        <v>5</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1074,8 +1138,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="4">
-        <f>C11/C10</f>
-        <v>0.2</v>
+        <v>7</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>14</v>
@@ -1087,6 +1150,11 @@
       </c>
       <c r="C13" s="3">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C14">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -1232,7 +1300,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="25.21875" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="35" customWidth="1"/>
@@ -1418,25 +1487,57 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
+    <row r="9" spans="1:8" ht="182.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="220.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
@@ -1589,7 +1690,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1599,7 +1700,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -1609,62 +1710,62 @@
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
         <v>59</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1821,73 +1922,73 @@
     </row>
     <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1912,7 +2013,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1920,7 +2021,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -1928,185 +2029,195 @@
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D7" s="13"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D10" s="13"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="D14" s="13"/>
+        <v>145</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="D15" s="13"/>
+        <v>145</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="D16" s="13"/>
+        <v>145</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="D17" s="13"/>
+        <v>145</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="D18" s="13"/>
+        <v>145</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="20" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="16" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2114,13 +2225,13 @@
         <v>44</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>